<commit_message>
feat: integrate real-time KPI dashboard, update README, and fix UI container width
</commit_message>
<xml_diff>
--- a/data/output/traceability_report.xlsx
+++ b/data/output/traceability_report.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E-E Traceability Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="E-E Traceability Report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat: finalize AI traceability agent MVP for demo
- Implemented real-time latency tracking and RAG context validation in LangGraph state.
- Updated LLM prompt to dynamically generate error categories for Pareto analysis.
- Expanded mock requirements dataset to simulate a production-scale dashboard.
- Restructured README.md with non-technical step-by-step UI guide and dashboard screenshots.
</commit_message>
<xml_diff>
--- a/data/output/traceability_report.xlsx
+++ b/data/output/traceability_report.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,11 +477,7 @@
           <t>CONFLICT</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>The requirement asks for a specific voltage (48V) that conflicts with the context specifying a different voltage (12V).</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -499,11 +495,151 @@
           <t>VALID</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>The requirement asks for a maximum power draw of 15A, which matches the context's maximum current capability of 15 Amp.</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REQ-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Battery_Management</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>VALID</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REQ-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Radar_Sensor</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>VALID</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REQ-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Body_Control_Module</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>VALID</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REQ-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Engine_ECU</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REQ-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ADAS_Domain_Controller</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>VALID</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>REQ-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Steering_ECU</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>VALID</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>REQ-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HVAC_Module</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>REQ-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Telematics_Unit</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>VALID</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: upgrade to multi-document RAG with metadata source tracking
Architectural Upgrades:
- UI: Enabled multi-PDF upload in Streamlit and updated API calls.
- API: Added /upload-pdfs endpoint to FastAPI to handle parallel file ingestion.
- RAG: Updated vector_store.py to attach exact filenames as ChromaDB metadata for precise source tracking. Fixed deprecated langchain import.
- Agent: Overhauled graph_agent.py prompts to enforce 'Exact Metric Matching' (preventing LLM metric hallucination) and extract source document names.
- Dashboard: Fixed Matplotlib memory leaks (ghosting charts) and added the 'Source Document' column to the raw analytics log.
- Testing: Updated mock requirements to validate across Gateway, BMS, and Radar specs.
</commit_message>
<xml_diff>
--- a/data/output/traceability_report.xlsx
+++ b/data/output/traceability_report.xlsx
@@ -45,12 +45,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -474,7 +474,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>CONFLICT</t>
+          <t>VALID</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -487,12 +487,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Infotainment_Display</t>
+          <t>ECU_Gateway</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>CONFLICT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -505,10 +505,10 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Battery_Management</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+          <t>Telematics_Unit</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>VALID</t>
         </is>
@@ -523,12 +523,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Radar_Sensor</t>
+          <t>Telematics_Unit</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>CONFLICT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -541,10 +541,10 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Body_Control_Module</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
+          <t>Battery_Management</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>VALID</t>
         </is>
@@ -559,10 +559,10 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Engine_ECU</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
+          <t>Battery_Management</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>CONFLICT</t>
         </is>
@@ -577,10 +577,10 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ADAS_Domain_Controller</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+          <t>Battery_Management</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>VALID</t>
         </is>
@@ -595,10 +595,10 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Steering_ECU</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+          <t>Radar_Sensor</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>VALID</t>
         </is>
@@ -613,12 +613,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HVAC_Module</t>
+          <t>Radar_Sensor</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>CONFLICT</t>
+          <t>VALID</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -631,12 +631,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Telematics_Unit</t>
+          <t>Radar_Sensor</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>VALID</t>
+          <t>CONFLICT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>

</xml_diff>